<commit_message>
Fix: Add manual profile data fetching fallback for creator tracking
Added fallback logic to manually fetch profile data when foreign key relationship is not yet established. This ensures "Recorded by" field works immediately without requiring SQL migrations.

Changes:
- Added manual profile fetching in all activity pages (inspections, varroa treatments/checks, feedings, harvests)
- Fetches profiles data separately if not automatically joined by Supabase
- Maps profile data to records using user_id lookup
- Added user_id field to all activity interfaces for type safety
- Fixed TypeScript errors by using proper type annotations instead of 'any'

The solution works both:
- Without foreign keys (using manual fetch)
- With foreign keys (using automatic Supabase join)

This provides immediate functionality while the SQL migrations can be run at convenience.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/external_references/approved_varroa_treatments_ireland_with_summary.xlsx
+++ b/external_references/approved_varroa_treatments_ireland_with_summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rico Zmarzly\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2a7d248e1c1b7c5c/Bees/Apps/beekeeper-app/external_references/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9857FFA9-3009-4D97-9D4A-E80F0FB484C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{9857FFA9-3009-4D97-9D4A-E80F0FB484C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C79F2FEA-240B-4822-BD32-4FF48B06C37B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -584,19 +584,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="64.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="32.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="28" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -622,7 +622,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -648,7 +648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -674,7 +674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -700,7 +700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
@@ -726,7 +726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>30</v>
       </c>
@@ -752,7 +752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>37</v>
       </c>
@@ -778,7 +778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>43</v>
       </c>
@@ -804,7 +804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>48</v>
       </c>
@@ -830,7 +830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>51</v>
       </c>
@@ -864,9 +864,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="79.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="66.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>55</v>
       </c>
@@ -877,7 +887,7 @@
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -900,7 +910,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -926,7 +936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -952,7 +962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -978,7 +988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -1004,7 +1014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -1030,7 +1040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -1056,7 +1066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -1082,7 +1092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -1108,7 +1118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>51</v>
       </c>
@@ -1134,42 +1144,42 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>63</v>
       </c>

</xml_diff>